<commit_message>
Ecosistemas V6: completar M27B1 y M9B1 con una capa complementaria
- Mueve 'ECOSISTEMAS M27B1_M9B1.zip' a datos/gis/ecosistemas_complemento_M27B1_M9B1.zip.
- El script acepta capas complementarias (--complemento o «complemento» en
  el nombre) que solo rellenan los vacíos de la capa base.
- Se regeneran láminas, Excel y GeoPackage: sin cobertura baja de 803.059 ha
  a 0.736 ha (bordes de M10B4 y M6B2-3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C1CwVqdF28RaTpFEmDe8sc
</commit_message>
<xml_diff>
--- a/mapas/salidas/IN_Piura_Ecosistemas_por_Bloque_V6.xlsx
+++ b/mapas/salidas/IN_Piura_Ecosistemas_por_Bloque_V6.xlsx
@@ -578,7 +578,7 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM), recorte a microcuencas (ecosistemas_microcuencas). Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
+          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM): recorte a microcuencas, completado en M27B1 y M9B1 con el recorte a esos bloques. Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
         <v/>
       </c>
       <c r="G9" s="6" t="n">
-        <v>187482.9</v>
+        <v>188280.249</v>
       </c>
       <c r="H9" s="8">
         <f>IF(N(G9)=0,"",E9/G9)</f>
@@ -685,7 +685,7 @@
         <v/>
       </c>
       <c r="G10" s="10" t="n">
-        <v>155862.921</v>
+        <v>155867.895</v>
       </c>
       <c r="H10" s="12">
         <f>IF(N(G10)=0,"",E10/G10)</f>
@@ -732,10 +732,14 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Sin información de ecosistema</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr"/>
+          <t>Bosque relicto montano de vertiente occidental</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Br-mvoc</t>
+        </is>
+      </c>
       <c r="D12" s="9">
         <f>COUNTIF(Bloque_Ecosistema!$F$9:$F$198,B12)</f>
         <v/>
@@ -748,7 +752,9 @@
         <f>E12/E$15</f>
         <v/>
       </c>
-      <c r="G12" s="10" t="n"/>
+      <c r="G12" s="10" t="n">
+        <v>6281.805</v>
+      </c>
       <c r="H12" s="12">
         <f>IF(N(G12)=0,"",E12/G12)</f>
         <v/>
@@ -760,12 +766,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Bosque relicto montano de vertiente occidental</t>
+          <t>Páramo</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Br-mvoc</t>
+          <t>Pa</t>
         </is>
       </c>
       <c r="D13" s="5">
@@ -781,7 +787,7 @@
         <v/>
       </c>
       <c r="G13" s="6" t="n">
-        <v>6281.805</v>
+        <v>3843.332</v>
       </c>
       <c r="H13" s="8">
         <f>IF(N(G13)=0,"",E13/G13)</f>
@@ -794,14 +800,10 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Páramo</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Pa</t>
-        </is>
-      </c>
+          <t>Sin información de ecosistema</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr"/>
       <c r="D14" s="9">
         <f>COUNTIF(Bloque_Ecosistema!$F$9:$F$198,B14)</f>
         <v/>
@@ -814,9 +816,7 @@
         <f>E14/E$15</f>
         <v/>
       </c>
-      <c r="G14" s="10" t="n">
-        <v>3843.332</v>
-      </c>
+      <c r="G14" s="10" t="n"/>
       <c r="H14" s="12">
         <f>IF(N(G14)=0,"",E14/G14)</f>
         <v/>
@@ -919,7 +919,7 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM), recorte a microcuencas (ecosistemas_microcuencas). Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
+          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM): recorte a microcuencas, completado en M27B1 y M9B1 con el recorte a esos bloques. Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Sin información de ecosistema</t>
+          <t>Bosque relicto montano de vertiente occidental</t>
         </is>
       </c>
       <c r="B12" s="10">
@@ -1045,7 +1045,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Bosque relicto montano de vertiente occidental</t>
+          <t>Páramo</t>
         </is>
       </c>
       <c r="B13" s="6">
@@ -1068,7 +1068,7 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Páramo</t>
+          <t>Sin información de ecosistema</t>
         </is>
       </c>
       <c r="B14" s="10">
@@ -1184,7 +1184,7 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM), recorte a microcuencas (ecosistemas_microcuencas). Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
+          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM): recorte a microcuencas, completado en M27B1 y M9B1 con el recorte a esos bloques. Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
         </is>
       </c>
     </row>
@@ -4381,13 +4381,17 @@
       </c>
       <c r="H81" s="5" t="inlineStr">
         <is>
-          <t>Sin información de ecosistema</t>
+          <t>Bosque estacionalmente seco de colina y montaña</t>
         </is>
       </c>
       <c r="I81" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J81" s="5" t="inlineStr"/>
+        <v>0.9889</v>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>Zona agrícola (1%)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
@@ -4422,17 +4426,13 @@
       </c>
       <c r="H82" s="9" t="inlineStr">
         <is>
-          <t>Sin información de ecosistema</t>
+          <t>Bosque estacionalmente seco de colina y montaña</t>
         </is>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0.9948</v>
-      </c>
-      <c r="J82" s="9" t="inlineStr">
-        <is>
-          <t>Bosque estacionalmente seco de colina y montaña (1%)</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J82" s="9" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n">
@@ -6402,7 +6402,7 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM), recorte a microcuencas (ecosistemas_microcuencas). Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
+          <t>Fuente: Ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM): recorte a microcuencas, completado en M27B1 y M9B1 con el recorte a esos bloques. Bloques V6, ANIN-DIME-SESDI 2026 (sin 74 y 75)</t>
         </is>
       </c>
     </row>
@@ -12067,12 +12067,16 @@
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>Sin información de ecosistema</t>
-        </is>
-      </c>
-      <c r="G123" s="5" t="inlineStr"/>
+          <t>Bosque estacionalmente seco de colina y montaña</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>Bes-cm</t>
+        </is>
+      </c>
       <c r="H123" s="6" t="n">
-        <v>448.804</v>
+        <v>443.83</v>
       </c>
       <c r="I123" s="7">
         <f>H123/SUMIF($B$9:$B$198,B123,$H$9:$H$198)</f>
@@ -12092,12 +12096,12 @@
       </c>
       <c r="B124" s="9" t="inlineStr">
         <is>
-          <t>M9B1</t>
+          <t>M27B1</t>
         </is>
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>C1096-Q9545</t>
+          <t>C1096-Q9557</t>
         </is>
       </c>
       <c r="D124" s="9" t="inlineStr">
@@ -12112,19 +12116,23 @@
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>Sin información de ecosistema</t>
-        </is>
-      </c>
-      <c r="G124" s="9" t="inlineStr"/>
+          <t>Zona agrícola</t>
+        </is>
+      </c>
+      <c r="G124" s="9" t="inlineStr">
+        <is>
+          <t>Agri</t>
+        </is>
+      </c>
       <c r="H124" s="10" t="n">
-        <v>353.518</v>
+        <v>4.974</v>
       </c>
       <c r="I124" s="11">
         <f>H124/SUMIF($B$9:$B$198,B124,$H$9:$H$198)</f>
         <v/>
       </c>
       <c r="J124" s="10" t="n">
-        <v>355.364</v>
+        <v>448.804</v>
       </c>
       <c r="K124" s="10">
         <f>I124*J124</f>
@@ -12166,7 +12174,7 @@
         </is>
       </c>
       <c r="H125" s="6" t="n">
-        <v>1.845</v>
+        <v>355.364</v>
       </c>
       <c r="I125" s="7">
         <f>H125/SUMIF($B$9:$B$198,B125,$H$9:$H$198)</f>
@@ -15816,7 +15824,7 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Capa de ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM), recorte a microcuencas (ecosistemas_microcuencas).</t>
+          <t>Capa de ecosistemas: Mapa Nacional de Ecosistemas del Perú, MINAM 2018 (R.M. N.° 440-2018-MINAM): recorte a microcuencas, completado en M27B1 y M9B1 con el recorte a esos bloques.</t>
         </is>
       </c>
     </row>

</xml_diff>